<commit_message>
Updated Changes for 30/07/26
</commit_message>
<xml_diff>
--- a/attendance_output.xlsx
+++ b/attendance_output.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pwcindia-my.sharepoint.com/personal/abhinandan_roy_pwc_com/Documents/Documents/work-in-sync/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_7B6912919781946FAD60C6F0505ED87656CD90E9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B53B62B-9963-4799-9D38-476441FB3D96}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_F9D88E4CA0A708CB99BA5B188FEA105138F77AC1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BC5700C-21D8-425C-9851-45FAC0E68CB1}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="29-07-26(1)" sheetId="1" r:id="rId1"/>
+    <sheet name="29-07-26(2)" sheetId="2" r:id="rId2"/>
+    <sheet name="29-07-26(3)" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="93">
   <si>
     <t>date</t>
   </si>
@@ -351,10 +353,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1516,4 +1514,1753 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F43"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="4" max="4" width="29" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" t="s">
+        <v>9</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" t="s">
+        <v>9</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33" t="s">
+        <v>9</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" t="s">
+        <v>9</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D38" t="s">
+        <v>18</v>
+      </c>
+      <c r="E38" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>6</v>
+      </c>
+      <c r="B39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" t="s">
+        <v>84</v>
+      </c>
+      <c r="D39" t="s">
+        <v>18</v>
+      </c>
+      <c r="E39" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" t="s">
+        <v>85</v>
+      </c>
+      <c r="C40" t="s">
+        <v>86</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>89</v>
+      </c>
+      <c r="C42" t="s">
+        <v>90</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43" t="s">
+        <v>91</v>
+      </c>
+      <c r="C43" t="s">
+        <v>92</v>
+      </c>
+      <c r="D43" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:F43"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="22.7265625" customWidth="1"/>
+    <col min="4" max="4" width="25.36328125" customWidth="1"/>
+    <col min="5" max="5" width="26.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" t="s">
+        <v>9</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" t="s">
+        <v>70</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" t="s">
+        <v>9</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33" t="s">
+        <v>9</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" t="s">
+        <v>9</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" t="s">
+        <v>9</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>6</v>
+      </c>
+      <c r="B38" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D38" t="s">
+        <v>18</v>
+      </c>
+      <c r="E38" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>6</v>
+      </c>
+      <c r="B39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" t="s">
+        <v>84</v>
+      </c>
+      <c r="D39" t="s">
+        <v>18</v>
+      </c>
+      <c r="E39" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" t="s">
+        <v>85</v>
+      </c>
+      <c r="C40" t="s">
+        <v>86</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>89</v>
+      </c>
+      <c r="C42" t="s">
+        <v>90</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42" t="s">
+        <v>9</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>6</v>
+      </c>
+      <c r="B43" t="s">
+        <v>91</v>
+      </c>
+      <c r="C43" t="s">
+        <v>92</v>
+      </c>
+      <c r="D43" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>